<commit_message>
Enhance Streamlit app with verified PDF export, base64 assets, and investor previews
</commit_message>
<xml_diff>
--- a/WEEKLY REPORT SPREADSHEET.xlsx
+++ b/WEEKLY REPORT SPREADSHEET.xlsx
@@ -1492,13 +1492,13 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>24329.85</v>
+        <v>24337.4</v>
       </c>
       <c r="C2" s="20" t="n">
-        <v>-36.15</v>
+        <v>-28.6</v>
       </c>
       <c r="D2" s="19" t="n">
-        <v>-0.0015</v>
+        <v>-0.0012</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>24630.4</v>
@@ -1519,13 +1519,13 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>57585.95</v>
+        <v>57638.9</v>
       </c>
       <c r="C3" s="20" t="n">
-        <v>94.84999999999999</v>
+        <v>147.8</v>
       </c>
       <c r="D3" s="19" t="n">
-        <v>0.0016</v>
+        <v>0.0026</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>58015.85</v>
@@ -1546,16 +1546,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>26261.4</v>
+        <v>26276.6</v>
       </c>
       <c r="C4" s="20" t="n">
-        <v>47.75</v>
+        <v>62.95</v>
       </c>
       <c r="D4" s="19" t="n">
-        <v>0.0018</v>
+        <v>0.0024</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>26299.05</v>
+        <v>26305.75</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>26051.75</v>
@@ -1573,13 +1573,13 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>77794.10000000001</v>
+        <v>77831.91</v>
       </c>
       <c r="C5" s="20" t="n">
-        <v>-215.15</v>
+        <v>-177.34</v>
       </c>
       <c r="D5" s="19" t="n">
-        <v>-0.0028</v>
+        <v>-0.0023</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>78757.39999999999</v>
@@ -1856,10 +1856,10 @@
         </is>
       </c>
       <c r="B2" s="20" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C2" s="20" t="n">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
@@ -1880,10 +1880,10 @@
         </is>
       </c>
       <c r="B3" s="20" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C3" s="20" t="n">
-        <v>243</v>
+        <v>254</v>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
@@ -3123,110 +3123,110 @@
     <row r="2" ht="22.5" customHeight="1" s="21">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>INDSWFTLAB</t>
+          <t>SRPL</t>
         </is>
       </c>
       <c r="B2" s="20" t="inlineStr">
         <is>
-          <t>INDSWFTLAB</t>
+          <t>SRPL</t>
         </is>
       </c>
       <c r="C2" s="20" t="inlineStr">
         <is>
-          <t>17-Aug-2026 14:42:46</t>
+          <t>17-Aug-2026 15:08:09</t>
         </is>
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
-          <t>Investor Presentation</t>
+          <t>Outcome of Board Meeting</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1" s="21">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>SIGMAADV</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B3" s="20" t="inlineStr">
         <is>
-          <t>SIGMAADV</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="C3" s="20" t="inlineStr">
         <is>
-          <t>17-Aug-2026 14:41:29</t>
+          <t>17-Aug-2026 15:06:38</t>
         </is>
       </c>
       <c r="D3" s="20" t="inlineStr">
         <is>
-          <t>General Updates</t>
+          <t>Shareholders meeting</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1" s="21">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>MUKANDLTD</t>
+          <t>SRPL</t>
         </is>
       </c>
       <c r="B4" s="20" t="inlineStr">
         <is>
-          <t>MUKANDLTD</t>
+          <t>SRPL</t>
         </is>
       </c>
       <c r="C4" s="20" t="inlineStr">
         <is>
-          <t>17-Aug-2026 14:41:21</t>
+          <t>17-Aug-2026 15:05:06</t>
         </is>
       </c>
       <c r="D4" s="20" t="inlineStr">
         <is>
-          <t>Credit Rating- Revision</t>
+          <t>Outcome of Board Meeting</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1" s="21">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="B5" s="20" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>GOODLUCK</t>
         </is>
       </c>
       <c r="C5" s="20" t="inlineStr">
         <is>
-          <t>17-Aug-2026 14:40:58</t>
+          <t>17-Aug-2026 15:04:25</t>
         </is>
       </c>
       <c r="D5" s="20" t="inlineStr">
         <is>
-          <t>Analysts/Institutional Investor Meet/Con. Call Updates</t>
+          <t>Record Date</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1" s="21">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>MOKSH</t>
+          <t>EXCELINDUS</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>MOKSH</t>
+          <t>EXCELINDUS</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>17-Aug-2026 14:38:50</t>
+          <t>17-Aug-2026 15:03:49</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Copy of Newspaper Publication</t>
+          <t>Investor Presentation</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(pipeline): add resilient yfinance fallback in Step 1 to eliminate Streamlit Cloud browser crash during live refresh
</commit_message>
<xml_diff>
--- a/WEEKLY REPORT SPREADSHEET.xlsx
+++ b/WEEKLY REPORT SPREADSHEET.xlsx
@@ -1492,13 +1492,13 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>24337.4</v>
+        <v>24287.65</v>
       </c>
       <c r="C2" s="20" t="n">
-        <v>-28.6</v>
+        <v>-78.34999999999999</v>
       </c>
       <c r="D2" s="19" t="n">
-        <v>-0.0012</v>
+        <v>-0.0032</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>24630.4</v>
@@ -1519,13 +1519,13 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>57638.9</v>
+        <v>57497.8</v>
       </c>
       <c r="C3" s="20" t="n">
-        <v>147.8</v>
+        <v>6.7</v>
       </c>
       <c r="D3" s="19" t="n">
-        <v>0.0026</v>
+        <v>0.0001</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>58015.85</v>
@@ -1546,16 +1546,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>26276.6</v>
+        <v>26217.15</v>
       </c>
       <c r="C4" s="20" t="n">
-        <v>62.95</v>
+        <v>3.5</v>
       </c>
       <c r="D4" s="19" t="n">
-        <v>0.0024</v>
+        <v>0.0001</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>26305.75</v>
+        <v>26322.55</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>26051.75</v>
@@ -1573,13 +1573,13 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>77831.91</v>
+        <v>77728.16</v>
       </c>
       <c r="C5" s="20" t="n">
-        <v>-177.34</v>
+        <v>-281.09</v>
       </c>
       <c r="D5" s="19" t="n">
-        <v>-0.0023</v>
+        <v>-0.0036</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>78757.39999999999</v>
@@ -1856,10 +1856,10 @@
         </is>
       </c>
       <c r="B2" s="20" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C2" s="20" t="n">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
@@ -1880,10 +1880,10 @@
         </is>
       </c>
       <c r="B3" s="20" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C3" s="20" t="n">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
@@ -3123,110 +3123,110 @@
     <row r="2" ht="22.5" customHeight="1" s="21">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>SRPL</t>
+          <t>MACPOWER</t>
         </is>
       </c>
       <c r="B2" s="20" t="inlineStr">
         <is>
-          <t>SRPL</t>
+          <t>MACPOWER</t>
         </is>
       </c>
       <c r="C2" s="20" t="inlineStr">
         <is>
-          <t>17-Aug-2026 15:08:09</t>
+          <t>17-Aug-2026 16:39:03</t>
         </is>
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
-          <t>Outcome of Board Meeting</t>
+          <t>Updates</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1" s="21">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>SUMEETINDS</t>
         </is>
       </c>
       <c r="B3" s="20" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>SUMEETINDS</t>
         </is>
       </c>
       <c r="C3" s="20" t="inlineStr">
         <is>
-          <t>17-Aug-2026 15:06:38</t>
+          <t>17-Aug-2026 16:38:54</t>
         </is>
       </c>
       <c r="D3" s="20" t="inlineStr">
         <is>
-          <t>Shareholders meeting</t>
+          <t>General Updates</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1" s="21">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>SRPL</t>
+          <t>NELCO</t>
         </is>
       </c>
       <c r="B4" s="20" t="inlineStr">
         <is>
-          <t>SRPL</t>
+          <t>NELCO</t>
         </is>
       </c>
       <c r="C4" s="20" t="inlineStr">
         <is>
-          <t>17-Aug-2026 15:05:06</t>
+          <t>17-Aug-2026 16:38:36</t>
         </is>
       </c>
       <c r="D4" s="20" t="inlineStr">
         <is>
-          <t>Outcome of Board Meeting</t>
+          <t>Copy of Newspaper Publication</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1" s="21">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>GOODLUCK</t>
+          <t>V2RETAIL</t>
         </is>
       </c>
       <c r="B5" s="20" t="inlineStr">
         <is>
-          <t>GOODLUCK</t>
+          <t>V2RETAIL</t>
         </is>
       </c>
       <c r="C5" s="20" t="inlineStr">
         <is>
-          <t>17-Aug-2026 15:04:25</t>
+          <t>17-Aug-2026 16:37:45</t>
         </is>
       </c>
       <c r="D5" s="20" t="inlineStr">
         <is>
-          <t>Record Date</t>
+          <t>Analysts/Institutional Investor Meet/Con. Call Updates</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1" s="21">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>EXCELINDUS</t>
+          <t>THEMISMED</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>EXCELINDUS</t>
+          <t>THEMISMED</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>17-Aug-2026 15:03:49</t>
+          <t>17-Aug-2026 16:37:39</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Investor Presentation</t>
+          <t>General Updates</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
style(typography): boost local PDF font sizes to 11.5px with refined vertical margins and zero footer overlap
</commit_message>
<xml_diff>
--- a/WEEKLY REPORT SPREADSHEET.xlsx
+++ b/WEEKLY REPORT SPREADSHEET.xlsx
@@ -1867,7 +1867,7 @@
         </is>
       </c>
       <c r="E2" s="20" t="n">
-        <v>20.56</v>
+        <v>20.53</v>
       </c>
       <c r="F2" s="20" t="n">
         <v>21.1</v>
@@ -1891,7 +1891,7 @@
         </is>
       </c>
       <c r="E3" s="20" t="n">
-        <v>22.94</v>
+        <v>22.91</v>
       </c>
       <c r="F3" s="20" t="n">
         <v>23.25</v>
@@ -2325,10 +2325,10 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>20.56</v>
+        <v>20.53</v>
       </c>
       <c r="C2" s="10" t="n">
-        <v>2.97</v>
+        <v>2.95</v>
       </c>
       <c r="D2" s="20" t="n">
         <v>21.1</v>
@@ -2351,10 +2351,10 @@
         </is>
       </c>
       <c r="B3" s="10" t="n">
-        <v>22.94</v>
+        <v>22.91</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>3.32</v>
+        <v>3.31</v>
       </c>
       <c r="D3" s="20" t="n">
         <v>23.25</v>
@@ -2403,10 +2403,10 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>20</v>
+        <v>19.65</v>
       </c>
       <c r="C5" s="10" t="n">
-        <v>5.52</v>
+        <v>5.42</v>
       </c>
       <c r="D5" s="20" t="n">
         <v>28.5</v>
@@ -3123,17 +3123,17 @@
     <row r="2" ht="22.5" customHeight="1" s="21">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>MACPOWER</t>
+          <t>YUKEN</t>
         </is>
       </c>
       <c r="B2" s="20" t="inlineStr">
         <is>
-          <t>MACPOWER</t>
+          <t>YUKEN</t>
         </is>
       </c>
       <c r="C2" s="20" t="inlineStr">
         <is>
-          <t>17-Aug-2026 16:39:03</t>
+          <t>17-Aug-2026 17:40:22</t>
         </is>
       </c>
       <c r="D2" s="20" t="inlineStr">
@@ -3145,88 +3145,88 @@
     <row r="3" ht="22.5" customHeight="1" s="21">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>SUMEETINDS</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B3" s="20" t="inlineStr">
         <is>
-          <t>SUMEETINDS</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="C3" s="20" t="inlineStr">
         <is>
-          <t>17-Aug-2026 16:38:54</t>
+          <t>17-Aug-2026 17:38:02</t>
         </is>
       </c>
       <c r="D3" s="20" t="inlineStr">
         <is>
-          <t>General Updates</t>
+          <t>News Verification</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1" s="21">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>NELCO</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B4" s="20" t="inlineStr">
         <is>
-          <t>NELCO</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="C4" s="20" t="inlineStr">
         <is>
-          <t>17-Aug-2026 16:38:36</t>
+          <t>17-Aug-2026 17:37:54</t>
         </is>
       </c>
       <c r="D4" s="20" t="inlineStr">
         <is>
-          <t>Copy of Newspaper Publication</t>
+          <t>News Verification</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1" s="21">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>V2RETAIL</t>
+          <t>PREMIERPOL</t>
         </is>
       </c>
       <c r="B5" s="20" t="inlineStr">
         <is>
-          <t>V2RETAIL</t>
+          <t>PREMIERPOL</t>
         </is>
       </c>
       <c r="C5" s="20" t="inlineStr">
         <is>
-          <t>17-Aug-2026 16:37:45</t>
+          <t>17-Aug-2026 17:37:46</t>
         </is>
       </c>
       <c r="D5" s="20" t="inlineStr">
         <is>
-          <t>Analysts/Institutional Investor Meet/Con. Call Updates</t>
+          <t>Spurt in Volume</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1" s="21">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>THEMISMED</t>
+          <t>OMINFRAL</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>THEMISMED</t>
+          <t>OMINFRAL</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>17-Aug-2026 16:37:39</t>
+          <t>17-Aug-2026 17:36:42</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>General Updates</t>
+          <t>Awarding of order(s)/contract(s)</t>
         </is>
       </c>
     </row>

</xml_diff>